<commit_message>
FA35-12-DL verwijderd uit alle 3 CSV's
580N/588N-56/-58.pdf gecontroleerd: dekken alleen bestaande maten
(-8/-10/-12/-16), geen nieuwe data mogelijk voor de -04/-06 gaten.
Ontbrekende_persgegevens.xlsx geregenereerd (142 -> 141).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUVA1TaPw9or4iDCMSTAyb
</commit_message>
<xml_diff>
--- a/Ontbrekende_persgegevens.xlsx
+++ b/Ontbrekende_persgegevens.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -679,17 +679,17 @@
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>FA35</t>
+          <t>0449</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>0449</t>
+          <t>431</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -699,7 +699,7 @@
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>7200</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -709,7 +709,7 @@
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>FA35</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
@@ -1311,7 +1311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5705,12 +5705,12 @@
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>FA35-12-DL</t>
+          <t>FA35-16</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>PARLOCK FIREARMOR R35 DN19 (19.1MM) 3/4 WP 350</t>
+          <t>PARLOCK FIREARMOR R35 DN25 (25.4MM) 1 WP 350</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
-          <t>FA35-12-DL</t>
+          <t>FA35-16</t>
         </is>
       </c>
       <c r="G128" s="5" t="inlineStr">
@@ -5742,12 +5742,12 @@
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>FA35-16</t>
+          <t>FA35-20</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>PARLOCK FIREARMOR R35 DN25 (25.4MM) 1 WP 350</t>
+          <t>PARLOCK FIREARMOR R35 DN31  (31.8MM) 1 WP 350</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>FA35-16</t>
+          <t>FA35-20</t>
         </is>
       </c>
       <c r="G129" s="5" t="inlineStr">
@@ -5779,12 +5779,12 @@
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>FA35-20</t>
+          <t>FA35-6</t>
         </is>
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>PARLOCK FIREARMOR R35 DN31  (31.8MM) 1 WP 350</t>
+          <t>PARLOCK FIREARMOR R35 DN10 (9.5MM) 3/8 WP 350</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
-          <t>FA35-20</t>
+          <t>FA35-6</t>
         </is>
       </c>
       <c r="G130" s="5" t="inlineStr">
@@ -5816,12 +5816,12 @@
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>FA35-6</t>
+          <t>FA35-8</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>PARLOCK FIREARMOR R35 DN10 (9.5MM) 3/8 WP 350</t>
+          <t>PARLOCK FIREARMOR R35 DN12 (12.7MM) 1/2 WP 350</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>FA35-6</t>
+          <t>FA35-8</t>
         </is>
       </c>
       <c r="G131" s="5" t="inlineStr">
@@ -5853,17 +5853,17 @@
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>FA35-8</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>PARLOCK FIREARMOR R35 DN12 (12.7MM) 1/2 WP 350</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>FA35</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -5873,34 +5873,30 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
-          <t>FA35-8</t>
-        </is>
-      </c>
-      <c r="G132" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
+          <t>P000199</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -5915,7 +5911,7 @@
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>P000199</t>
+          <t>20LNBL008000079</t>
         </is>
       </c>
       <c r="G133" s="5" t="inlineStr"/>
@@ -5923,17 +5919,17 @@
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -5948,7 +5944,7 @@
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>20LNBL008000079</t>
+          <t>P000201</t>
         </is>
       </c>
       <c r="G134" s="5" t="inlineStr"/>
@@ -5956,7 +5952,7 @@
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
@@ -5966,7 +5962,7 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -5981,7 +5977,7 @@
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>P000201</t>
+          <t>P000196</t>
         </is>
       </c>
       <c r="G135" s="5" t="inlineStr"/>
@@ -5989,7 +5985,7 @@
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="B136" s="5" t="inlineStr">
@@ -5999,7 +5995,7 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
@@ -6014,7 +6010,7 @@
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
-          <t>P000196</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="G136" s="5" t="inlineStr"/>
@@ -6022,7 +6018,7 @@
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
@@ -6032,7 +6028,7 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
@@ -6047,7 +6043,7 @@
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>P000197</t>
         </is>
       </c>
       <c r="G137" s="5" t="inlineStr"/>
@@ -6055,17 +6051,17 @@
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 12X19MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 12X19MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
@@ -6080,7 +6076,7 @@
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>P000197</t>
+          <t>20LNBL013000079</t>
         </is>
       </c>
       <c r="G138" s="5" t="inlineStr"/>
@@ -6088,17 +6084,17 @@
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 13X19MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 13X19MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
@@ -6113,7 +6109,7 @@
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>20LNBL013000079</t>
+          <t>P000198</t>
         </is>
       </c>
       <c r="G139" s="5" t="inlineStr"/>
@@ -6121,17 +6117,17 @@
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 19X28MM</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>PARKER HOSE 1/8″</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 19X28MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
@@ -6141,12 +6137,12 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
-          <t>P000198</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="G140" s="5" t="inlineStr"/>
@@ -6154,17 +6150,17 @@
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>PDH-2</t>
+          <t>R35TC-40</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>PARKER HOSE 1/8″</t>
+          <t>R13 TC 63.5MM (21/2) DN63 IN-/OUT. SKIVE W.P. 350 BAR</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>PDH</t>
+          <t>R35TC</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -6179,20 +6175,24 @@
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="G141" s="5" t="inlineStr"/>
+          <t>R35TC-40</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>R35TC-40</t>
+          <t>R35TC-48</t>
         </is>
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>R13 TC 63.5MM (21/2) DN63 IN-/OUT. SKIVE W.P. 350 BAR</t>
+          <t>R13 TC 76MM (3) DN76 IN-/OUT. SKIVE W.P. 350 BAR</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
@@ -6212,7 +6212,7 @@
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
-          <t>R35TC-40</t>
+          <t>RS35TC-48</t>
         </is>
       </c>
       <c r="G142" s="5" t="inlineStr">
@@ -6221,45 +6221,8 @@
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="5" t="inlineStr">
-        <is>
-          <t>R35TC-48</t>
-        </is>
-      </c>
-      <c r="B143" s="5" t="inlineStr">
-        <is>
-          <t>R13 TC 76MM (3) DN76 IN-/OUT. SKIVE W.P. 350 BAR</t>
-        </is>
-      </c>
-      <c r="C143" s="5" t="inlineStr">
-        <is>
-          <t>R35TC</t>
-        </is>
-      </c>
-      <c r="D143" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E143" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F143" s="5" t="inlineStr">
-        <is>
-          <t>RS35TC-48</t>
-        </is>
-      </c>
-      <c r="G143" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G143"/>
+  <autoFilter ref="A1:G142"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
FA35/221FR/431/R35TC-40-48/563TJ: persgegevens aangevuld uit nieuwe Parker perslijsten
- FA35-6/-8 (VS), FA35-12/-16/-20 (V4): 2-delig, Huls=Pilaar=code,
  waarden bevestigd tegen bestaande 100V4-16/-20-koppelingen.
- 221FR-8/-12: 1-delig Huls 26, Werkdruk 35 (extrapolatie familie).
- 431-4/-6/-8/-12/-16: 1-delig Huls 43, bron in inches, omgerekend naar mm.
- R35TC-40/-48: laatste 2 gaten in de R35TC-familie (100V6-40/-48, V6).
- 0563TJ-4/-6/-8: 1-delig Huls 55 (Tough Jacket-stijl), bron in inches;
  55-serie gekozen omdat dit exact overeenkomt met bestaande 0590TJ-06/-08.

Alle nieuwe waarden gelijk toegepast in Staal en RVS (crimp-/schilgegevens
zijn materiaalonafhankelijk per instructie gebruiker).

Ontbrekende_persgegevens.xlsx geregenereerd (141 -> 124).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUVA1TaPw9or4iDCMSTAyb
</commit_message>
<xml_diff>
--- a/Ontbrekende_persgegevens.xlsx
+++ b/Ontbrekende_persgegevens.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F81"/>
+  <dimension ref="B2:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>7200</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -699,27 +699,27 @@
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>FA35</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
@@ -729,7 +729,7 @@
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
+          <t>540N</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
@@ -739,57 +739,57 @@
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
+          <t>0503</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
+          <t>0560</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>0503</t>
+          <t>0347</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>0560</t>
+          <t>0427</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>0563TJ</t>
+          <t>0441</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>0347</t>
+          <t>0447</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -799,7 +799,7 @@
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>0427</t>
+          <t>5155</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -809,7 +809,7 @@
     <row r="33">
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>0441</t>
+          <t>518C</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -819,7 +819,7 @@
     <row r="34">
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>0447</t>
+          <t>580N</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -829,7 +829,7 @@
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>221FR</t>
+          <t>588N</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -839,57 +839,57 @@
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
+          <t>0315</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
+          <t>0328</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
+          <t>0442</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
+          <t>0480</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>R35TC</t>
+          <t>0561</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>0315</t>
+          <t>2245D</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -899,7 +899,7 @@
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>0328</t>
+          <t>2248D</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
@@ -909,7 +909,7 @@
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>0442</t>
+          <t>2380M</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -919,7 +919,7 @@
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>0480</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -929,7 +929,7 @@
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>0561</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -939,7 +939,7 @@
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
+          <t>526BA</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
@@ -949,7 +949,7 @@
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>540P</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
@@ -959,7 +959,7 @@
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
@@ -969,7 +969,7 @@
     <row r="49">
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
@@ -979,7 +979,7 @@
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>7200N</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -989,7 +989,7 @@
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
+          <t>811</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
@@ -999,7 +999,7 @@
     <row r="52">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
+          <t>881</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
@@ -1009,7 +1009,7 @@
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
@@ -1019,7 +1019,7 @@
     <row r="54">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
@@ -1029,7 +1029,7 @@
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
@@ -1039,7 +1039,7 @@
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>AIR10MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="C56" s="5" t="n">
@@ -1049,7 +1049,7 @@
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="C57" s="5" t="n">
@@ -1059,7 +1059,7 @@
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR13MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="C58" s="5" t="n">
@@ -1069,7 +1069,7 @@
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR13MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="C59" s="5" t="n">
@@ -1079,7 +1079,7 @@
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="C60" s="5" t="n">
@@ -1089,7 +1089,7 @@
     <row r="61">
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="C61" s="5" t="n">
@@ -1099,7 +1099,7 @@
     <row r="62">
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR19MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="C62" s="5" t="n">
@@ -1109,7 +1109,7 @@
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>AIR19MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -1119,7 +1119,7 @@
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>AIR19MMGRIJS</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -1129,7 +1129,7 @@
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="C65" s="5" t="n">
@@ -1139,7 +1139,7 @@
     <row r="66">
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>AIR25MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="C66" s="5" t="n">
@@ -1149,7 +1149,7 @@
     <row r="67">
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="C67" s="5" t="n">
@@ -1159,7 +1159,7 @@
     <row r="68">
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="C68" s="5" t="n">
@@ -1169,7 +1169,7 @@
     <row r="69">
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="C69" s="5" t="n">
@@ -1179,7 +1179,7 @@
     <row r="70">
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="C70" s="5" t="n">
@@ -1189,7 +1189,7 @@
     <row r="71">
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="C71" s="5" t="n">
@@ -1199,7 +1199,7 @@
     <row r="72">
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="C72" s="5" t="n">
@@ -1209,7 +1209,7 @@
     <row r="73">
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="C73" s="5" t="n">
@@ -1219,7 +1219,7 @@
     <row r="74">
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="C74" s="5" t="n">
@@ -1229,7 +1229,7 @@
     <row r="75">
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="C75" s="5" t="n">
@@ -1239,60 +1239,10 @@
     <row r="76">
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="C76" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1311,7 +1261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2932,17 +2882,17 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>0563TJ-4</t>
+          <t>0620-06</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>TOUGH JACKET HOSE SAE 100R17 210 BAR</t>
+          <t>MTR NYLAFLOW HOSE</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>0563TJ</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2952,34 +2902,30 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Flowtech</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>563TJ-4</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
+          <t>0620-06</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>0563TJ-6</t>
+          <t>0620-08</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>TOUGH JACKET HOSE SAE 100R17 210 BAR</t>
+          <t>MTR NYLAFLOW HOSE</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>0563TJ</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2989,34 +2935,30 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Flowtech</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>563TJ-6</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
+          <t>0620-08</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>0563TJ-8</t>
+          <t>0620-10</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>TOUGH JACKET HOSE SAE 100R17 210 BAR</t>
+          <t>MTR NYLAFLOW HOSE</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>0563TJ</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -3026,24 +2968,20 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Flowtech</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>563TJ-8</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
+          <t>0620-10</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -3068,7 +3006,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -3076,7 +3014,7 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -3086,7 +3024,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -3101,7 +3039,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -3109,7 +3047,7 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -3119,7 +3057,7 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -3134,7 +3072,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -3142,7 +3080,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
@@ -3152,7 +3090,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -3167,7 +3105,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -3175,7 +3113,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -3200,7 +3138,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr"/>
@@ -3208,32 +3146,32 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>0811-04-316</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0811</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Flowtech</t>
+          <t>Polyfluor plastics</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>801AGP316DN06</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -3241,32 +3179,32 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>0811-05-316</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0811</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Flowtech</t>
+          <t>Polyfluor plastics</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>801AGP316dn08</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -3274,32 +3212,32 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>0811-06A</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE</t>
+          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0811</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Flowtech</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>T1AB010</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -3307,12 +3245,12 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>0811-04-316</t>
+          <t>0811-08A</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
+          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -3327,12 +3265,12 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Polyfluor plastics</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>801AGP316DN06</t>
+          <t>T1AB012</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -3340,12 +3278,12 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>0811-05-316</t>
+          <t>0811-10</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -3360,25 +3298,29 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Polyfluor plastics</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>801AGP316dn08</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr"/>
+          <t>M290016</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>0811-06A</t>
+          <t>0811-12</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -3398,20 +3340,24 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>T1AB010</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr"/>
+          <t>TB1020</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>0811-08A</t>
+          <t>0811-16</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3426,30 +3372,34 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>T1AB012</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="inlineStr"/>
+          <t>M290025</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>0811-10</t>
+          <t>0815-04</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>0811</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -3459,34 +3409,34 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>M290016</t>
+          <t>TCB1E006L</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>0811-12</t>
+          <t>0815-05</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>0811</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -3501,29 +3451,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>TB1020</t>
+          <t>TCB1E008</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>138</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>0811-16</t>
+          <t>0815-08A</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>0811</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -3538,24 +3488,20 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>M290025</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+          <t>M293013</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>0815-04</t>
+          <t>0815-16A</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -3570,119 +3516,115 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>TCB1E006L</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>172</t>
-        </is>
-      </c>
+          <t>M293025</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>0815-05</t>
+          <t>2245D-03V32</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
+          <t>MTR POLYFLEX SLANG</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>2245D</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>TCB1E008</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
-      </c>
+          <t>2245D-03V32</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>0815-08A</t>
+          <t>2248D-05V32-TC</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
+          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
-        </is>
-      </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>2248D</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>M293013</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr"/>
+          <t>2248D-05V32-TC</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>1035</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>0815-16A</t>
+          <t>2380M-04V30W</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>PARKER POLYFLEX SLANG BLACK</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>2380M</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>M293025</t>
+          <t>2380M-04V30W</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -3690,17 +3632,17 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>221FR-12</t>
+          <t>2648N-32V80</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>5/8 MARINE FUEL</t>
+          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>221FR</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -3715,25 +3657,29 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>221FR-12</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="inlineStr"/>
+          <t>2648N-32V80</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>221FR-8</t>
+          <t>510A-4</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>13/32 MARINE FUEL</t>
+          <t>PARFLEX 510A-4 DN06</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>221FR</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -3748,7 +3694,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>221FR-8</t>
+          <t>510A-4</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -3756,17 +3702,17 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SLANG</t>
+          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
+          <t>5155</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3781,7 +3727,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -3789,17 +3735,17 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
+          <t>5155-5</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
+          <t>PARFLEX 5155-5 DN08</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>5155</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -3814,34 +3760,30 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>1035</t>
-        </is>
-      </c>
+          <t>5155-5</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
+          <t>518C-04</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>PARKER POLYFLEX SLANG BLACK</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>518C</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3851,30 +3793,34 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr"/>
+          <t>518C-4</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
+          <t>518C-06</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>518C</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3884,29 +3830,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
+          <t>518C-6</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>155</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>431-12</t>
+          <t>526BA-4</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>MTR COMPACT NO-SKIVE HOSE</t>
+          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>526BA</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -3921,25 +3867,29 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>431-12</t>
-        </is>
-      </c>
-      <c r="G75" s="5" t="inlineStr"/>
+          <t>526BA-4</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>413,7</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>431-16</t>
+          <t>540N-2</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>MTR COMPACT NO-SKIVE HOSE</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>540N</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -3954,7 +3904,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>431-16</t>
+          <t>540N-2</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -3962,22 +3912,22 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>431-4</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>MTR COMPACT NO-SKIVE HOSE</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>431</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>540N</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3987,7 +3937,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>431-4</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr"/>
@@ -3995,22 +3945,22 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>431-6</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>MTR COMPACT NO-SKIVE HOSE</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>431</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>540N</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -4020,7 +3970,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>431-6</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -4028,22 +3978,22 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>431-8</t>
+          <t>540N-8</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>MTR COMPACT NO-SKIVE HOSE</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>431</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>540N</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -4053,7 +4003,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>431-8</t>
+          <t>540N-8-DL</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr"/>
@@ -4061,17 +4011,17 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 510A-4 DN06</t>
+          <t>PARFLEX-SCHLAUCH DN12 H</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>540P</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -4086,7 +4036,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr"/>
@@ -4094,17 +4044,17 @@
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>56DH-2</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
+          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -4119,7 +4069,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>56DH-2</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr"/>
@@ -4127,17 +4077,17 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
+          <t>575XN-8</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 5155-5 DN08</t>
+          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -4152,30 +4102,34 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr"/>
+          <t>575XN-8</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>344,7</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>518C-04</t>
+          <t>580N-04</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
+          <t>PARFLEX HOSE 580N-4</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
-        </is>
-      </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>580N</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -4185,34 +4139,30 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>518C-4</t>
-        </is>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
-        <is>
-          <t>190</t>
-        </is>
-      </c>
+          <t>580N-4</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>518C-06</t>
+          <t>580N-06</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
+          <t>PARFLEX HOSE 580N-6</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
-        </is>
-      </c>
-      <c r="D84" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>580N</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -4222,34 +4172,30 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>518C-6</t>
-        </is>
-      </c>
-      <c r="G84" s="5" t="inlineStr">
-        <is>
-          <t>155</t>
-        </is>
-      </c>
+          <t>580N-6</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
+          <t>588N-06</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
+          <t>MTR PARFLEX SLANG R8 588N-6</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>588N</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -4259,34 +4205,30 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
-        </is>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>413,7</t>
-        </is>
-      </c>
+          <t>588N-6</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
+          <t>588N-4</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>MTR PARFLEX SLANG R8</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>588N</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -4296,7 +4238,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
+          <t>588N-4</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr"/>
@@ -4304,116 +4246,128 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
+          <t>7200-04</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>HYDR. HOSE 700 BAR</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="inlineStr"/>
+          <t>VHP-DN06-0412</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
+          <t>7200-04TWIN</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>HYDR. HOSE 700 BAR TWIN</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
-        </is>
-      </c>
-      <c r="D88" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr"/>
+          <t>VHPD-DN06-1412</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>540N-8</t>
+          <t>7200-06</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>HYDR. HOSE 700 BAR</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
-        </is>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>540N-8-DL</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="inlineStr"/>
+          <t>VHP-DN10-0414</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
+          <t>7200-06LGR</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX-SCHLAUCH DN12 H</t>
+          <t>HYDR. HOSE 700 BAR LIME GREEN</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
+          <t>7200</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -4423,30 +4377,34 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr"/>
+          <t>VHP-DN10-0404 LIOME GREEN</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
+          <t>7200-06ORA</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
+          <t>HYDR. HOSE 700 BAR ORANGE</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>7200</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -4456,30 +4414,34 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr"/>
+          <t>VHP-DN10-0404 ORANGE</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
+          <t>7200N-04</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
+          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>7200N</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -4489,34 +4451,34 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
+          <t>VHP-DN06-0462</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>344,7</t>
+          <t>700</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>580N-04</t>
+          <t>811-56</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-4</t>
+          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
+          <t>811</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -4526,12 +4488,12 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>580N-4</t>
+          <t>14A-56</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr"/>
@@ -4539,17 +4501,17 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>580N-06</t>
+          <t>811S-32</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-6</t>
+          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
+          <t>811S</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -4564,30 +4526,34 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>580N-6</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="inlineStr"/>
+          <t>811S-32</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>588N-06</t>
+          <t>811S-40</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8 588N-6</t>
+          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
-        </is>
-      </c>
-      <c r="D95" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>811S</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -4597,30 +4563,34 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>588N-6</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="inlineStr"/>
+          <t>811S-40</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
+          <t>811S-48</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8</t>
+          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>811S</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -4630,25 +4600,29 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
-        </is>
-      </c>
-      <c r="G96" s="5" t="inlineStr"/>
+          <t>811S-48</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>7200-04</t>
+          <t>811S-56</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR</t>
+          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>811S</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -4658,71 +4632,63 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0412</t>
-        </is>
-      </c>
-      <c r="G97" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>811S-56</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>7200-04TWIN</t>
+          <t>811S-64</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR TWIN</t>
+          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>811S</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>VHPD-DN06-1412</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>811S-64</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>7200-06</t>
+          <t>811S-80</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR</t>
+          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>811S</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
@@ -4732,71 +4698,63 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0414</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>811S-80</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>7200-06LGR</t>
+          <t>811S-96</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR LIME GREEN</t>
+          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
-        </is>
-      </c>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>811S</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0404 LIOME GREEN</t>
-        </is>
-      </c>
-      <c r="G100" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>811S-96</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>7200-06ORA</t>
+          <t>881-40</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR ORANGE</t>
+          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>881</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -4806,34 +4764,34 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0404 ORANGE</t>
+          <t>881-40</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>7200N-04</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
+          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -4843,34 +4801,30 @@
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0462</t>
-        </is>
-      </c>
-      <c r="G102" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>P002228</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>811-56</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -4880,12 +4834,12 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>14A-56</t>
+          <t>P002231</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr"/>
@@ -4893,17 +4847,17 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -4913,123 +4867,111 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
-        </is>
-      </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>P002208</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
+          <t>AIR10MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 10x3,5</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR10MMGEEL 15 BAR</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>P001869</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR13MM</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>P002211</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>AIR13MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 13x3,5</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR13MMGEEL 15 BAR</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>10LU15013YEL406</t>
         </is>
       </c>
       <c r="G107" s="5" t="inlineStr"/>
@@ -5037,32 +4979,32 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>AIR13MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 13x23 mm</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR13MMGEEL 20 BAR</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>10LU20013YOO406</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr"/>
@@ -5070,32 +5012,32 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR16MM</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Arbon</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
+          <t>5941625 L=50 mtr.</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr"/>
@@ -5103,32 +5045,32 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR19MM</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Arbon</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
+          <t>5941929-NOBRA AIR L=20 mtr</t>
         </is>
       </c>
       <c r="G110" s="5" t="inlineStr"/>
@@ -5136,17 +5078,17 @@
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
+          <t>AIR19MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 19x4,5</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>AIR19MMGEEL 15 BAR</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -5156,34 +5098,30 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
-        </is>
-      </c>
-      <c r="G111" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>10LU15019YEL406</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR19MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
+          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 19x31 mm</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR19MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -5198,7 +5136,7 @@
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>P002228</t>
+          <t>P001903</t>
         </is>
       </c>
       <c r="G112" s="5" t="inlineStr"/>
@@ -5206,17 +5144,17 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR19MMGRIJS</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>LUCHTSLANG UNIVERSEL 3/4 GRIJS</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR19MMGRIJS</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -5231,7 +5169,7 @@
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>P002231</t>
+          <t>AIR19MMGRIJS</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr"/>
@@ -5239,17 +5177,17 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -5264,7 +5202,7 @@
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>P002208</t>
+          <t>P002223</t>
         </is>
       </c>
       <c r="G114" s="5" t="inlineStr"/>
@@ -5272,17 +5210,17 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR25MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 10x3,5</t>
+          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 25x37 mm</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR25MMGEEL 20 BAR</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -5297,7 +5235,7 @@
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>P001869</t>
+          <t>10LU20025YOO406</t>
         </is>
       </c>
       <c r="G115" s="5" t="inlineStr"/>
@@ -5305,17 +5243,17 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -5330,7 +5268,7 @@
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>P002211</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="G116" s="5" t="inlineStr"/>
@@ -5338,17 +5276,17 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 13x3,5</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -5363,7 +5301,7 @@
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>10LU15013YEL406</t>
+          <t>P000199</t>
         </is>
       </c>
       <c r="G117" s="5" t="inlineStr"/>
@@ -5371,17 +5309,17 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 13x23 mm</t>
+          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -5396,7 +5334,7 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>10LU20013YOO406</t>
+          <t>20LNBL008000079</t>
         </is>
       </c>
       <c r="G118" s="5" t="inlineStr"/>
@@ -5404,17 +5342,17 @@
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -5424,12 +5362,12 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>Arbon</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>5941625 L=50 mtr.</t>
+          <t>P000201</t>
         </is>
       </c>
       <c r="G119" s="5" t="inlineStr"/>
@@ -5437,17 +5375,17 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -5457,12 +5395,12 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>Arbon</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>5941929-NOBRA AIR L=20 mtr</t>
+          <t>P000196</t>
         </is>
       </c>
       <c r="G120" s="5" t="inlineStr"/>
@@ -5470,17 +5408,17 @@
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 19x4,5</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -5495,7 +5433,7 @@
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>10LU15019YEL406</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr"/>
@@ -5503,17 +5441,17 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 19x31 mm</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -5528,7 +5466,7 @@
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
-          <t>P001903</t>
+          <t>P000197</t>
         </is>
       </c>
       <c r="G122" s="5" t="inlineStr"/>
@@ -5536,17 +5474,17 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG UNIVERSEL 3/4 GRIJS</t>
+          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -5561,7 +5499,7 @@
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>20LNBL013000079</t>
         </is>
       </c>
       <c r="G123" s="5" t="inlineStr"/>
@@ -5569,17 +5507,17 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
@@ -5594,7 +5532,7 @@
       </c>
       <c r="F124" s="5" t="inlineStr">
         <is>
-          <t>P002223</t>
+          <t>P000198</t>
         </is>
       </c>
       <c r="G124" s="5" t="inlineStr"/>
@@ -5602,17 +5540,17 @@
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 25x37 mm</t>
+          <t>PARKER HOSE 1/8″</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -5622,607 +5560,18 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>10LU20025YOO406</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="G125" s="5" t="inlineStr"/>
     </row>
-    <row r="126">
-      <c r="A126" s="5" t="inlineStr">
-        <is>
-          <t>AIR38MM</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
-        <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>AIR38MM</t>
-        </is>
-      </c>
-      <c r="D126" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F126" s="5" t="inlineStr">
-        <is>
-          <t>AIR38MM</t>
-        </is>
-      </c>
-      <c r="G126" s="5" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="5" t="inlineStr">
-        <is>
-          <t>FA35-12</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr">
-        <is>
-          <t>PARLOCK FIREARMOR R35 DN19 (19.1MM) 3/4 WP 350</t>
-        </is>
-      </c>
-      <c r="C127" s="5" t="inlineStr">
-        <is>
-          <t>FA35</t>
-        </is>
-      </c>
-      <c r="D127" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E127" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F127" s="5" t="inlineStr">
-        <is>
-          <t>FA35-12</t>
-        </is>
-      </c>
-      <c r="G127" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t>FA35-16</t>
-        </is>
-      </c>
-      <c r="B128" s="5" t="inlineStr">
-        <is>
-          <t>PARLOCK FIREARMOR R35 DN25 (25.4MM) 1 WP 350</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>FA35</t>
-        </is>
-      </c>
-      <c r="D128" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E128" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F128" s="5" t="inlineStr">
-        <is>
-          <t>FA35-16</t>
-        </is>
-      </c>
-      <c r="G128" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="5" t="inlineStr">
-        <is>
-          <t>FA35-20</t>
-        </is>
-      </c>
-      <c r="B129" s="5" t="inlineStr">
-        <is>
-          <t>PARLOCK FIREARMOR R35 DN31  (31.8MM) 1 WP 350</t>
-        </is>
-      </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>FA35</t>
-        </is>
-      </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E129" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F129" s="5" t="inlineStr">
-        <is>
-          <t>FA35-20</t>
-        </is>
-      </c>
-      <c r="G129" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="5" t="inlineStr">
-        <is>
-          <t>FA35-6</t>
-        </is>
-      </c>
-      <c r="B130" s="5" t="inlineStr">
-        <is>
-          <t>PARLOCK FIREARMOR R35 DN10 (9.5MM) 3/8 WP 350</t>
-        </is>
-      </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>FA35</t>
-        </is>
-      </c>
-      <c r="D130" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E130" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F130" s="5" t="inlineStr">
-        <is>
-          <t>FA35-6</t>
-        </is>
-      </c>
-      <c r="G130" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>FA35-8</t>
-        </is>
-      </c>
-      <c r="B131" s="5" t="inlineStr">
-        <is>
-          <t>PARLOCK FIREARMOR R35 DN12 (12.7MM) 1/2 WP 350</t>
-        </is>
-      </c>
-      <c r="C131" s="5" t="inlineStr">
-        <is>
-          <t>FA35</t>
-        </is>
-      </c>
-      <c r="D131" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E131" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F131" s="5" t="inlineStr">
-        <is>
-          <t>FA35-8</t>
-        </is>
-      </c>
-      <c r="G131" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 06X12MM</t>
-        </is>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C132" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 06X12MM</t>
-        </is>
-      </c>
-      <c r="D132" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E132" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F132" s="5" t="inlineStr">
-        <is>
-          <t>P000199</t>
-        </is>
-      </c>
-      <c r="G132" s="5" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X13MM</t>
-        </is>
-      </c>
-      <c r="B133" s="5" t="inlineStr">
-        <is>
-          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
-        </is>
-      </c>
-      <c r="C133" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X13MM</t>
-        </is>
-      </c>
-      <c r="D133" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E133" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F133" s="5" t="inlineStr">
-        <is>
-          <t>20LNBL008000079</t>
-        </is>
-      </c>
-      <c r="G133" s="5" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X14MM</t>
-        </is>
-      </c>
-      <c r="B134" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C134" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X14MM</t>
-        </is>
-      </c>
-      <c r="D134" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E134" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F134" s="5" t="inlineStr">
-        <is>
-          <t>P000201</t>
-        </is>
-      </c>
-      <c r="G134" s="5" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MM</t>
-        </is>
-      </c>
-      <c r="B135" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C135" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MM</t>
-        </is>
-      </c>
-      <c r="D135" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E135" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F135" s="5" t="inlineStr">
-        <is>
-          <t>P000196</t>
-        </is>
-      </c>
-      <c r="G135" s="5" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="B136" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C136" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="D136" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E136" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F136" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="G136" s="5" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="B137" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C137" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="D137" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E137" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F137" s="5" t="inlineStr">
-        <is>
-          <t>P000197</t>
-        </is>
-      </c>
-      <c r="G137" s="5" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="B138" s="5" t="inlineStr">
-        <is>
-          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
-        </is>
-      </c>
-      <c r="C138" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="D138" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E138" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F138" s="5" t="inlineStr">
-        <is>
-          <t>20LNBL013000079</t>
-        </is>
-      </c>
-      <c r="G138" s="5" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="B139" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C139" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="D139" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E139" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F139" s="5" t="inlineStr">
-        <is>
-          <t>P000198</t>
-        </is>
-      </c>
-      <c r="G139" s="5" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="B140" s="5" t="inlineStr">
-        <is>
-          <t>PARKER HOSE 1/8″</t>
-        </is>
-      </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="D140" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E140" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F140" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="G140" s="5" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="5" t="inlineStr">
-        <is>
-          <t>R35TC-40</t>
-        </is>
-      </c>
-      <c r="B141" s="5" t="inlineStr">
-        <is>
-          <t>R13 TC 63.5MM (21/2) DN63 IN-/OUT. SKIVE W.P. 350 BAR</t>
-        </is>
-      </c>
-      <c r="C141" s="5" t="inlineStr">
-        <is>
-          <t>R35TC</t>
-        </is>
-      </c>
-      <c r="D141" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E141" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F141" s="5" t="inlineStr">
-        <is>
-          <t>R35TC-40</t>
-        </is>
-      </c>
-      <c r="G141" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="5" t="inlineStr">
-        <is>
-          <t>R35TC-48</t>
-        </is>
-      </c>
-      <c r="B142" s="5" t="inlineStr">
-        <is>
-          <t>R13 TC 76MM (3) DN76 IN-/OUT. SKIVE W.P. 350 BAR</t>
-        </is>
-      </c>
-      <c r="C142" s="5" t="inlineStr">
-        <is>
-          <t>R35TC</t>
-        </is>
-      </c>
-      <c r="D142" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E142" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F142" s="5" t="inlineStr">
-        <is>
-          <t>RS35TC-48</t>
-        </is>
-      </c>
-      <c r="G142" s="5" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G142"/>
+  <autoFilter ref="A1:G125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
IMM-coderingen vervangen door Geeve Perslijst; RVS 4SP-fix teruggedraaid; 10 artikelen verwijderd
- Ontdekt dat Geeve Perslijst_2018.pdf de oorspronkelijke bron is van
  de RVS 4SP-Persmaten (0441/0442) - de PH-perslijst-fix van twee
  rondes geleden overschreef die per abuis. Teruggedraaid, met een
  echte correctie op dash-20 (54,3, niet 51,2 of 52,6).
- 0446 (4SH) en 0447-32/0480-32 (R15): IMM-Huls (004N-xx/0013-xx)
  vervangen door Geeve Perslijst Z-serie (34000-xx/Z34000-xxRVS resp.
  Z37000-32/Z37000-32RVS), Pilaar 30-serie.
- 0447-10: IMM-waarde verwijderd zonder vervanging (Geeve Perslijst
  dekt dash-10 niet) - weer een open gat, bewust.
- 10 artikelen verwijderd (AIR-luchtslangen, 7200-serie): 949 -> 939.

Ontbrekende_persgegevens.xlsx geregenereerd (113 -> 104).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUVA1TaPw9or4iDCMSTAyb
</commit_message>
<xml_diff>
--- a/Ontbrekende_persgegevens.xlsx
+++ b/Ontbrekende_persgegevens.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F71"/>
+  <dimension ref="B2:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>949</v>
+        <v>939</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -679,17 +679,17 @@
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -699,7 +699,7 @@
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -709,7 +709,7 @@
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
+          <t>540N</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
@@ -719,17 +719,17 @@
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
+          <t>0503</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>0503</t>
+          <t>0560</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
@@ -739,17 +739,17 @@
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>0560</t>
+          <t>0347</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>0347</t>
+          <t>0427</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
@@ -759,7 +759,7 @@
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>0427</t>
+          <t>5155</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
@@ -769,7 +769,7 @@
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
+          <t>518C</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -779,7 +779,7 @@
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
+          <t>580N</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
@@ -789,7 +789,7 @@
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
+          <t>588N</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -799,7 +799,7 @@
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
+          <t>7200</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -829,7 +829,7 @@
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>0561</t>
+          <t>0447</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -839,7 +839,7 @@
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
+          <t>0561</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -849,7 +849,7 @@
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>2245D</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
@@ -859,7 +859,7 @@
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
+          <t>2248D</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
@@ -869,7 +869,7 @@
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
+          <t>2380M</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
@@ -879,7 +879,7 @@
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
@@ -889,7 +889,7 @@
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -899,7 +899,7 @@
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
+          <t>526BA</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
@@ -909,7 +909,7 @@
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>540P</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -919,7 +919,7 @@
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -929,7 +929,7 @@
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -939,7 +939,7 @@
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>7200N</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
@@ -949,7 +949,7 @@
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>811</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
@@ -959,7 +959,7 @@
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>881</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
@@ -969,7 +969,7 @@
     <row r="49">
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
@@ -979,7 +979,7 @@
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -989,7 +989,7 @@
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
@@ -1009,7 +1009,7 @@
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
@@ -1019,7 +1019,7 @@
     <row r="54">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
@@ -1029,7 +1029,7 @@
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
@@ -1039,7 +1039,7 @@
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="C56" s="5" t="n">
@@ -1049,7 +1049,7 @@
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="C57" s="5" t="n">
@@ -1059,7 +1059,7 @@
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="C58" s="5" t="n">
@@ -1069,7 +1069,7 @@
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="C59" s="5" t="n">
@@ -1079,7 +1079,7 @@
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="C60" s="5" t="n">
@@ -1089,7 +1089,7 @@
     <row r="61">
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="C61" s="5" t="n">
@@ -1099,7 +1099,7 @@
     <row r="62">
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="C62" s="5" t="n">
@@ -1109,7 +1109,7 @@
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -1119,7 +1119,7 @@
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -1129,70 +1129,10 @@
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="C65" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MM</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="C69" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="C71" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1211,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1736,40 +1676,44 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>0501-04</t>
+          <t>0447-10</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>RUBBER HOSE WITH TEXTILE 1TE LAYER (R6)</t>
+          <t>R15-DN16 (5/8) IN-/OUT. SKIVE W.P. 420 BAR</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>0501</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>0447</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>JB Hydraulics</t>
+          <t>Interpump</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>20-600-06</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
+          <t>TFDR015-10</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>0501-06</t>
+          <t>0501-04</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1794,7 +1738,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>20-600-10</t>
+          <t>20-600-06</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -1802,7 +1746,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>0501-08</t>
+          <t>0501-06</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1827,7 +1771,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>20-600-13</t>
+          <t>20-600-10</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr"/>
@@ -1835,7 +1779,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>0501-10</t>
+          <t>0501-08</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1855,12 +1799,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Interpump</t>
+          <t>JB Hydraulics</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>TFS0006I10</t>
+          <t>20-600-13</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -1868,7 +1812,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>0501-12</t>
+          <t>0501-10</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1888,12 +1832,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>JB Hydraulics</t>
+          <t>Interpump</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>20-600-20</t>
+          <t>TFS0006I10</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -1901,7 +1845,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>0501-16</t>
+          <t>0501-12</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1921,12 +1865,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Interpump</t>
+          <t>JB Hydraulics</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>TFS0006I16</t>
+          <t>20-600-20</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr"/>
@@ -1934,32 +1878,32 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>0503-20</t>
+          <t>0501-16</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>RUBBER HOSE WITH TEXTILE 2 LAYER 3TE</t>
+          <t>RUBBER HOSE WITH TEXTILE 1TE LAYER (R6)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>0503</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>0501</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Interpump</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>SLMW-06-20</t>
+          <t>TFS0006I16</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -1967,7 +1911,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>0503-24</t>
+          <t>0503-20</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1987,12 +1931,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Eriks</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>TE 0338</t>
+          <t>SLMW-06-20</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -2000,7 +1944,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>0503-32</t>
+          <t>0503-24</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2020,12 +1964,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Eriks</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>48000</t>
+          <t>TE 0338</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -2033,32 +1977,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>0511-12</t>
+          <t>0503-32</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 19X29</t>
+          <t>RUBBER HOSE WITH TEXTILE 2 LAYER 3TE</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>0511</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>0503</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>P001279</t>
+          <t>48000</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -2066,12 +2010,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>0511-16</t>
+          <t>0511-12</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 25X35</t>
+          <t>SUCTION AND RETURN HOSE 19X29</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -2091,7 +2035,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>P001280</t>
+          <t>P001279</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>
@@ -2099,12 +2043,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>0511-20</t>
+          <t>0511-16</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 32X42</t>
+          <t>SUCTION AND RETURN HOSE 25X35</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -2124,7 +2068,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>P001284</t>
+          <t>P001280</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
@@ -2132,12 +2076,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>0511-24</t>
+          <t>0511-20</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 38X50</t>
+          <t>SUCTION AND RETURN HOSE 32X42</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -2157,7 +2101,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>P001286</t>
+          <t>P001284</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -2165,12 +2109,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>0511-32</t>
+          <t>0511-24</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 51X62</t>
+          <t>SUCTION AND RETURN HOSE 38X50</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2190,7 +2134,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>P001291</t>
+          <t>P001286</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -2198,12 +2142,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>0511-40</t>
+          <t>0511-32</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 63X76</t>
+          <t>SUCTION AND RETURN HOSE 51X62</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -2211,9 +2155,9 @@
           <t>0511</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2223,7 +2167,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>P001295</t>
+          <t>P001291</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -2231,12 +2175,12 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>0511-48</t>
+          <t>0511-40</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 76X90</t>
+          <t>SUCTION AND RETURN HOSE 63X76</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -2256,7 +2200,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>P002545</t>
+          <t>P001295</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr"/>
@@ -2264,12 +2208,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>0511-64</t>
+          <t>0511-48</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 102X118</t>
+          <t>SUCTION AND RETURN HOSE 76X90</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -2289,7 +2233,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>P001274</t>
+          <t>P002545</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr"/>
@@ -2297,17 +2241,17 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>0560-04</t>
+          <t>0511-64</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SAE100R1 560-4</t>
+          <t>SUCTION AND RETURN HOSE 102X118</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0560</t>
+          <t>0511</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2317,12 +2261,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>560-4</t>
+          <t>P001274</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -2330,12 +2274,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>0560-06</t>
+          <t>0560-04</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SAE100R1 560-6</t>
+          <t>MTR POLYFLEX SAE100R1 560-4</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2355,7 +2299,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>560-6</t>
+          <t>560-4</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr"/>
@@ -2363,12 +2307,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>0560-08-08</t>
+          <t>0560-06</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX TWINSLANG 1/2 SAE100R1 560-8-8</t>
+          <t>MTR POLYFLEX SAE100R1 560-6</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2388,7 +2332,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>560-8-8</t>
+          <t>560-6</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -2396,17 +2340,17 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>0561-08</t>
+          <t>0560-08-08</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TRELLJET 561 8 L100</t>
+          <t>MTR POLYFLEX TWINSLANG 1/2 SAE100R1 560-8-8</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>0561</t>
+          <t>0560</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2416,12 +2360,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Trelleborg</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>561-08</t>
+          <t>560-8-8</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -2429,17 +2373,17 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>0561-08</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE</t>
+          <t>TRELLJET 561 8 L100</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0561</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2449,12 +2393,12 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Flowtech</t>
+          <t>Trelleborg</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>561-08</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -2462,7 +2406,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0620-06</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -2487,7 +2431,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0620-06</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -2495,7 +2439,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0620-08</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -2520,7 +2464,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0620-08</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -2528,7 +2472,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0620-10</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2553,7 +2497,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0620-10</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -2561,7 +2505,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2571,7 +2515,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2586,7 +2530,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -2594,7 +2538,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2619,7 +2563,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr"/>
@@ -2627,7 +2571,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2652,7 +2596,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -2660,7 +2604,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2685,7 +2629,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -2693,32 +2637,32 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>0811-04-316</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
+          <t>MTR NYLAFLOW HOSE</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>0811</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>0628</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Polyfluor plastics</t>
+          <t>Flowtech</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>801AGP316DN06</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -2726,7 +2670,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>0811-05-316</t>
+          <t>0811-04-316</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2751,7 +2695,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>801AGP316dn08</t>
+          <t>801AGP316DN06</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -2759,12 +2703,12 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>0811-06A</t>
+          <t>0811-05-316</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -2779,12 +2723,12 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Polyfluor plastics</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>T1AB010</t>
+          <t>801AGP316dn08</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -2792,7 +2736,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>0811-08A</t>
+          <t>0811-06A</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2817,7 +2761,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>T1AB012</t>
+          <t>T1AB010</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -2825,12 +2769,12 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>0811-10</t>
+          <t>0811-08A</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
+          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -2845,29 +2789,25 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>M290016</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
+          <t>T1AB012</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>0811-12</t>
+          <t>0811-10</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -2882,29 +2822,29 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>TB1020</t>
+          <t>M290016</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>114</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>0811-16</t>
+          <t>0811-12</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -2919,34 +2859,34 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>M290025</t>
+          <t>TB1020</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>0815-04</t>
+          <t>0811-16</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
+          <t>0811</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -2956,29 +2896,29 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>TCB1E006L</t>
+          <t>M290025</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>0815-05</t>
+          <t>0815-04</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -2998,24 +2938,24 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>TCB1E008</t>
+          <t>TCB1E006L</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>0815-08A</t>
+          <t>0815-05</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -3030,25 +2970,29 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>M293013</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr"/>
+          <t>TCB1E008</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>0815-16A</t>
+          <t>0815-08A</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -3068,7 +3012,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>M293025</t>
+          <t>M293013</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr"/>
@@ -3076,32 +3020,32 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
+          <t>0815-16A</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SLANG</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0815</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
+          <t>M293025</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -3109,17 +3053,17 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
+          <t>2245D-03V32</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
+          <t>MTR POLYFLEX SLANG</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>2245D</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -3134,29 +3078,25 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>1035</t>
-        </is>
-      </c>
+          <t>2245D-03V32</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
+          <t>2248D-05V32-TC</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>PARKER POLYFLEX SLANG BLACK</t>
+          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
+          <t>2248D</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -3171,25 +3111,29 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr"/>
+          <t>2248D-05V32-TC</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>1035</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
+          <t>2380M-04V30W</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
+          <t>PARKER POLYFLEX SLANG BLACK</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
+          <t>2380M</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -3204,29 +3148,25 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>2380M-04V30W</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
+          <t>2648N-32V80</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 510A-4 DN06</t>
+          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -3241,25 +3181,29 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr"/>
+          <t>2648N-32V80</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>510A-4</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
+          <t>PARFLEX 510A-4 DN06</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -3274,7 +3218,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>510A-4</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -3282,12 +3226,12 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 5155-5 DN08</t>
+          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3307,7 +3251,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -3315,22 +3259,22 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>518C-04</t>
+          <t>5155-5</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
+          <t>PARFLEX 5155-5 DN08</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>5155</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -3340,24 +3284,20 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>518C-4</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>190</t>
-        </is>
-      </c>
+          <t>5155-5</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>518C-06</t>
+          <t>518C-04</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -3377,34 +3317,34 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>518C-6</t>
+          <t>518C-4</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>190</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
+          <t>518C-06</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>518C</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -3414,29 +3354,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
+          <t>518C-6</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>413,7</t>
+          <t>155</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
+          <t>526BA-4</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
+          <t>526BA</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3451,15 +3391,19 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr"/>
+          <t>526BA-4</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>413,7</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
+          <t>540N-2</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -3472,9 +3416,9 @@
           <t>540N</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -3484,7 +3428,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
+          <t>540N-2</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -3492,7 +3436,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -3517,7 +3461,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -3525,7 +3469,7 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>540N-8</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
@@ -3550,7 +3494,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>540N-8-DL</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -3558,22 +3502,22 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
+          <t>540N-8</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX-SCHLAUCH DN12 H</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>540N</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -3583,7 +3527,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
+          <t>540N-8-DL</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr"/>
@@ -3591,17 +3535,17 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
+          <t>PARFLEX-SCHLAUCH DN12 H</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>540P</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -3616,7 +3560,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -3624,17 +3568,17 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
+          <t>56DH-2</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
+          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3649,29 +3593,25 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr">
-        <is>
-          <t>344,7</t>
-        </is>
-      </c>
+          <t>56DH-2</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>580N-04</t>
+          <t>575XN-8</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-4</t>
+          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -3686,20 +3626,24 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>580N-4</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr"/>
+          <t>575XN-8</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>344,7</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>580N-06</t>
+          <t>580N-04</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-6</t>
+          <t>PARFLEX HOSE 580N-4</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3719,7 +3663,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>580N-6</t>
+          <t>580N-4</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -3727,22 +3671,22 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>588N-06</t>
+          <t>580N-06</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8 588N-6</t>
+          <t>PARFLEX HOSE 580N-6</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>580N</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3752,7 +3696,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>588N-6</t>
+          <t>580N-6</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr"/>
@@ -3760,12 +3704,12 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
+          <t>588N-06</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8</t>
+          <t>MTR PARFLEX SLANG R8 588N-6</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -3785,7 +3729,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
+          <t>588N-6</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -3793,49 +3737,45 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>7200-04</t>
+          <t>588N-4</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR</t>
+          <t>MTR PARFLEX SLANG R8</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>588N</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0412</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>588N-4</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>7200-04TWIN</t>
+          <t>7200-04</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR TWIN</t>
+          <t>HYDR. HOSE 700 BAR</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -3843,9 +3783,9 @@
           <t>7200</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3855,7 +3795,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>VHPD-DN06-1412</t>
+          <t>VHP-DN06-0412</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -3904,17 +3844,17 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>7200-06LGR</t>
+          <t>7200N-04</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR LIME GREEN</t>
+          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>7200N</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3929,7 +3869,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0404 LIOME GREEN</t>
+          <t>VHP-DN06-0462</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -3941,17 +3881,17 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>7200-06ORA</t>
+          <t>811-56</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR ORANGE</t>
+          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
+          <t>811</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -3961,34 +3901,30 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0404 ORANGE</t>
-        </is>
-      </c>
-      <c r="G80" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>14A-56</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>7200N-04</t>
+          <t>811S-32</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
+          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>811S</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -3998,62 +3934,66 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0462</t>
+          <t>811S-32</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>811-56</t>
+          <t>811S-40</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>811</t>
-        </is>
-      </c>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>811S</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>14A-56</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr"/>
+          <t>811S-40</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
+          <t>811S-48</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -4061,9 +4001,9 @@
           <t>811S</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -4073,7 +4013,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
+          <t>811S-48</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -4085,12 +4025,12 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
+          <t>811S-56</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -4110,24 +4050,20 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
-        </is>
-      </c>
-      <c r="G84" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>811S-56</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
+          <t>811S-64</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -4147,24 +4083,20 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
-        </is>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>811S-64</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>811S-80</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -4184,7 +4116,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>811S-80</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr"/>
@@ -4192,12 +4124,12 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>811S-96</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -4217,7 +4149,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>811S-96</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr"/>
@@ -4225,22 +4157,22 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
+          <t>881-40</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>881</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -4250,40 +4182,44 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr"/>
+          <t>881-40</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>AIR06MM</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
+          <t>P002228</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr"/>
@@ -4291,17 +4227,17 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -4311,34 +4247,30 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>P002231</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -4353,7 +4285,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>P002228</t>
+          <t>P002208</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr"/>
@@ -4361,17 +4293,17 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -4386,7 +4318,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>P002231</t>
+          <t>P002211</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr"/>
@@ -4394,17 +4326,17 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -4414,12 +4346,12 @@
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Arbon</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>P002208</t>
+          <t>5941625 L=50 mtr.</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr"/>
@@ -4427,17 +4359,17 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 10x3,5</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>AIR10MMGEEL 15 BAR</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -4447,12 +4379,12 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Arbon</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>P001869</t>
+          <t>5941929-NOBRA AIR L=20 mtr</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr"/>
@@ -4460,17 +4392,17 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -4485,7 +4417,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>P002211</t>
+          <t>P002223</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr"/>
@@ -4493,17 +4425,17 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 13x3,5</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 15 BAR</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -4518,7 +4450,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>10LU15013YEL406</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr"/>
@@ -4526,17 +4458,17 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 13x23 mm</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>AIR13MMGEEL 20 BAR</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -4551,7 +4483,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>10LU20013YOO406</t>
+          <t>P000199</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr"/>
@@ -4559,17 +4491,17 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -4579,12 +4511,12 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Arbon</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>5941625 L=50 mtr.</t>
+          <t>20LNBL008000079</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr"/>
@@ -4592,17 +4524,17 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -4612,12 +4544,12 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>Arbon</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>5941929-NOBRA AIR L=20 mtr</t>
+          <t>P000201</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr"/>
@@ -4625,17 +4557,17 @@
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/15 YELLOW ø 19x4,5</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 15 BAR</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -4650,7 +4582,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>10LU15019YEL406</t>
+          <t>P000196</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr"/>
@@ -4658,17 +4590,17 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 19x31 mm</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGEEL 20 BAR</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -4683,7 +4615,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>P001903</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr"/>
@@ -4691,17 +4623,17 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG UNIVERSEL 3/4 GRIJS</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -4716,7 +4648,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>AIR19MMGRIJS</t>
+          <t>P000197</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr"/>
@@ -4724,17 +4656,17 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -4749,7 +4681,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>P002223</t>
+          <t>20LNBL013000079</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr"/>
@@ -4757,17 +4689,17 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE UNIVERSAL/20-YELLOW ø 25x37 mm</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>AIR25MMGEEL 20 BAR</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -4782,7 +4714,7 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>10LU20025YOO406</t>
+          <t>P000198</t>
         </is>
       </c>
       <c r="G104" s="5" t="inlineStr"/>
@@ -4790,17 +4722,17 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>PARKER HOSE 1/8″</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -4810,315 +4742,18 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="G105" s="5" t="inlineStr"/>
     </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 06X12MM</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C106" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 06X12MM</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>P000199</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X13MM</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="inlineStr">
-        <is>
-          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X13MM</t>
-        </is>
-      </c>
-      <c r="D107" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F107" s="5" t="inlineStr">
-        <is>
-          <t>20LNBL008000079</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X14MM</t>
-        </is>
-      </c>
-      <c r="B108" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C108" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 08X14MM</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E108" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F108" s="5" t="inlineStr">
-        <is>
-          <t>P000201</t>
-        </is>
-      </c>
-      <c r="G108" s="5" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MM</t>
-        </is>
-      </c>
-      <c r="B109" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MM</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F109" s="5" t="inlineStr">
-        <is>
-          <t>P000196</t>
-        </is>
-      </c>
-      <c r="G109" s="5" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="B110" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C110" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="D110" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F110" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 10X16MMRED</t>
-        </is>
-      </c>
-      <c r="G110" s="5" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="B111" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 12X19MM</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E111" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F111" s="5" t="inlineStr">
-        <is>
-          <t>P000197</t>
-        </is>
-      </c>
-      <c r="G111" s="5" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 13X19MM</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>20LNBL013000079</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>NOBELAIR 19X28MM</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>Peters</t>
-        </is>
-      </c>
-      <c r="F113" s="5" t="inlineStr">
-        <is>
-          <t>P000198</t>
-        </is>
-      </c>
-      <c r="G113" s="5" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="B114" s="5" t="inlineStr">
-        <is>
-          <t>PARKER HOSE 1/8″</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="D114" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E114" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F114" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="G114" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G114"/>
+  <autoFilter ref="A1:G105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
0447-10 hersteld met Geeve Z34000-10-notatie
Vorige ronde per abuis leeggemaakt bij het verwijderen van IMM-codes.
De onderliggende meetwaarden (29,5/15,0/47,0mm, uit IMM-crimpchart)
zijn geldig gebleven - alleen de Huls-naam is nu Z34000-10 (Staal) /
Z34000-10RVS (RVS), Pilaar 30, consistent met de rest van de familie.

Ontbrekende_persgegevens.xlsx geregenereerd (104 -> 103).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DUVA1TaPw9or4iDCMSTAyb
</commit_message>
<xml_diff>
--- a/Ontbrekende_persgegevens.xlsx
+++ b/Ontbrekende_persgegevens.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F65"/>
+  <dimension ref="B2:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>0447</t>
+          <t>0561</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -839,7 +839,7 @@
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>0561</t>
+          <t>2245D</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -849,7 +849,7 @@
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
+          <t>2248D</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
@@ -859,7 +859,7 @@
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>2380M</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
@@ -869,7 +869,7 @@
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
@@ -879,7 +879,7 @@
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
@@ -889,7 +889,7 @@
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>526BA</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -899,7 +899,7 @@
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
+          <t>540P</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
@@ -909,7 +909,7 @@
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -919,7 +919,7 @@
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -929,7 +929,7 @@
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>7200N</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -939,7 +939,7 @@
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>811</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
@@ -949,7 +949,7 @@
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>881</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
@@ -959,7 +959,7 @@
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
@@ -969,7 +969,7 @@
     <row r="49">
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
@@ -979,7 +979,7 @@
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -989,7 +989,7 @@
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
@@ -999,7 +999,7 @@
     <row r="52">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
@@ -1009,7 +1009,7 @@
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
@@ -1019,7 +1019,7 @@
     <row r="54">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
@@ -1029,7 +1029,7 @@
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
@@ -1039,7 +1039,7 @@
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="C56" s="5" t="n">
@@ -1049,7 +1049,7 @@
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="C57" s="5" t="n">
@@ -1059,7 +1059,7 @@
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="C58" s="5" t="n">
@@ -1069,7 +1069,7 @@
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="C59" s="5" t="n">
@@ -1079,7 +1079,7 @@
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="C60" s="5" t="n">
@@ -1089,7 +1089,7 @@
     <row r="61">
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="C61" s="5" t="n">
@@ -1099,7 +1099,7 @@
     <row r="62">
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 12X19MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="C62" s="5" t="n">
@@ -1109,7 +1109,7 @@
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 13X19MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -1119,20 +1119,10 @@
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 19X28MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1151,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1676,44 +1666,40 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>0447-10</t>
+          <t>0501-04</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>R15-DN16 (5/8) IN-/OUT. SKIVE W.P. 420 BAR</t>
+          <t>RUBBER HOSE WITH TEXTILE 1TE LAYER (R6)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>0447</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0501</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Interpump</t>
+          <t>JB Hydraulics</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>TFDR015-10</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>420</t>
-        </is>
-      </c>
+          <t>20-600-06</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>0501-04</t>
+          <t>0501-06</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1738,7 +1724,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>20-600-06</t>
+          <t>20-600-10</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -1746,7 +1732,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>0501-06</t>
+          <t>0501-08</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1771,7 +1757,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>20-600-10</t>
+          <t>20-600-13</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr"/>
@@ -1779,7 +1765,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>0501-08</t>
+          <t>0501-10</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1799,12 +1785,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>JB Hydraulics</t>
+          <t>Interpump</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>20-600-13</t>
+          <t>TFS0006I10</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -1812,7 +1798,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>0501-10</t>
+          <t>0501-12</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1832,12 +1818,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Interpump</t>
+          <t>JB Hydraulics</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>TFS0006I10</t>
+          <t>20-600-20</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -1845,7 +1831,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>0501-12</t>
+          <t>0501-16</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1865,12 +1851,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>JB Hydraulics</t>
+          <t>Interpump</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>20-600-20</t>
+          <t>TFS0006I16</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr"/>
@@ -1878,32 +1864,32 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>0501-16</t>
+          <t>0503-20</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>RUBBER HOSE WITH TEXTILE 1TE LAYER (R6)</t>
+          <t>RUBBER HOSE WITH TEXTILE 2 LAYER 3TE</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>0501</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>0503</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Interpump</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>TFS0006I16</t>
+          <t>SLMW-06-20</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -1911,7 +1897,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>0503-20</t>
+          <t>0503-24</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1931,12 +1917,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Eriks</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>SLMW-06-20</t>
+          <t>TE 0338</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -1944,7 +1930,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>0503-24</t>
+          <t>0503-32</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1964,12 +1950,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Eriks</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>TE 0338</t>
+          <t>48000</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -1977,32 +1963,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>0503-32</t>
+          <t>0511-12</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>RUBBER HOSE WITH TEXTILE 2 LAYER 3TE</t>
+          <t>SUCTION AND RETURN HOSE 19X29</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>0503</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>0511</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>48000</t>
+          <t>P001279</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -2010,12 +1996,12 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>0511-12</t>
+          <t>0511-16</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 19X29</t>
+          <t>SUCTION AND RETURN HOSE 25X35</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -2035,7 +2021,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>P001279</t>
+          <t>P001280</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr"/>
@@ -2043,12 +2029,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>0511-16</t>
+          <t>0511-20</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 25X35</t>
+          <t>SUCTION AND RETURN HOSE 32X42</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -2068,7 +2054,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>P001280</t>
+          <t>P001284</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
@@ -2076,12 +2062,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>0511-20</t>
+          <t>0511-24</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 32X42</t>
+          <t>SUCTION AND RETURN HOSE 38X50</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -2101,7 +2087,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>P001284</t>
+          <t>P001286</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -2109,12 +2095,12 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>0511-24</t>
+          <t>0511-32</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 38X50</t>
+          <t>SUCTION AND RETURN HOSE 51X62</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -2134,7 +2120,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>P001286</t>
+          <t>P001291</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -2142,12 +2128,12 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>0511-32</t>
+          <t>0511-40</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 51X62</t>
+          <t>SUCTION AND RETURN HOSE 63X76</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -2155,9 +2141,9 @@
           <t>0511</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2167,7 +2153,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>P001291</t>
+          <t>P001295</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -2175,12 +2161,12 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>0511-40</t>
+          <t>0511-48</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 63X76</t>
+          <t>SUCTION AND RETURN HOSE 76X90</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -2200,7 +2186,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>P001295</t>
+          <t>P002545</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr"/>
@@ -2208,12 +2194,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>0511-48</t>
+          <t>0511-64</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 76X90</t>
+          <t>SUCTION AND RETURN HOSE 102X118</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -2233,7 +2219,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>P002545</t>
+          <t>P001274</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr"/>
@@ -2241,17 +2227,17 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>0511-64</t>
+          <t>0560-04</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>SUCTION AND RETURN HOSE 102X118</t>
+          <t>MTR POLYFLEX SAE100R1 560-4</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0511</t>
+          <t>0560</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2261,12 +2247,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>P001274</t>
+          <t>560-4</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -2274,12 +2260,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>0560-04</t>
+          <t>0560-06</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SAE100R1 560-4</t>
+          <t>MTR POLYFLEX SAE100R1 560-6</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2299,7 +2285,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>560-4</t>
+          <t>560-6</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr"/>
@@ -2307,12 +2293,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>0560-06</t>
+          <t>0560-08-08</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SAE100R1 560-6</t>
+          <t>MTR POLYFLEX TWINSLANG 1/2 SAE100R1 560-8-8</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2332,7 +2318,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>560-6</t>
+          <t>560-8-8</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -2340,17 +2326,17 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>0560-08-08</t>
+          <t>0561-08</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX TWINSLANG 1/2 SAE100R1 560-8-8</t>
+          <t>TRELLJET 561 8 L100</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>0560</t>
+          <t>0561</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2360,12 +2346,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Trelleborg</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>560-8-8</t>
+          <t>561-08</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -2373,17 +2359,17 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>0561-08</t>
+          <t>0620-06</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>TRELLJET 561 8 L100</t>
+          <t>MTR NYLAFLOW HOSE</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>0561</t>
+          <t>0620</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2393,12 +2379,12 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Trelleborg</t>
+          <t>Flowtech</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>561-08</t>
+          <t>0620-06</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -2406,7 +2392,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>0620-08</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -2431,7 +2417,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>0620-06</t>
+          <t>0620-08</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -2439,7 +2425,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0620-10</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -2464,7 +2450,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>0620-08</t>
+          <t>0620-10</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -2472,7 +2458,7 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2497,7 +2483,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>0620-10</t>
+          <t>0620-12</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -2505,7 +2491,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2515,7 +2501,7 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>0620</t>
+          <t>0628</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2530,7 +2516,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>0620-12</t>
+          <t>0628-04</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -2538,7 +2524,7 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2563,7 +2549,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>0628-04</t>
+          <t>0628-05</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr"/>
@@ -2571,7 +2557,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2596,7 +2582,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>0628-05</t>
+          <t>0628-06</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -2604,7 +2590,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -2629,7 +2615,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>0628-06</t>
+          <t>0628-08</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -2637,32 +2623,32 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>0811-04-316</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>0628</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>0811</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Flowtech</t>
+          <t>Polyfluor plastics</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>0628-08</t>
+          <t>801AGP316DN06</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -2670,7 +2656,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>0811-04-316</t>
+          <t>0811-05-316</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -2695,7 +2681,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>801AGP316DN06</t>
+          <t>801AGP316dn08</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -2703,12 +2689,12 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>0811-05-316</t>
+          <t>0811-06A</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST 316L BRAID</t>
+          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -2723,12 +2709,12 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Polyfluor plastics</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>801AGP316dn08</t>
+          <t>T1AB010</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -2736,7 +2722,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>0811-06A</t>
+          <t>0811-08A</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2761,7 +2747,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>T1AB010</t>
+          <t>T1AB012</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -2769,12 +2755,12 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>0811-08A</t>
+          <t>0811-10</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -2789,25 +2775,29 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>T1AB012</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr"/>
+          <t>M290016</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>0811-10</t>
+          <t>0811-12</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 114 BAR</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -2822,29 +2812,29 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>M290016</t>
+          <t>TB1020</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>0811-12</t>
+          <t>0811-16</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 103 BAR</t>
+          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -2859,34 +2849,34 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>TB1020</t>
+          <t>M290025</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>0811-16</t>
+          <t>0815-04</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>SMOOTH, BIG BORE PTFE HOSE, WITH ST/ST BRAID W.P. 80 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>0811</t>
+          <t>0815</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -2896,29 +2886,29 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Xtraflex</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>M290025</t>
+          <t>TCB1E006L</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>0815-04</t>
+          <t>0815-05</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 172 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -2938,24 +2928,24 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>TCB1E006L</t>
+          <t>TCB1E008</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>138</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>0815-05</t>
+          <t>0815-08A</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID W.P. 138 BAR</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -2970,29 +2960,25 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Xtraflex</t>
+          <t>Dicsa</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>TCB1E008</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
-      </c>
+          <t>M293013</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>0815-08A</t>
+          <t>0815-16A</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTISTATIC</t>
+          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -3012,7 +2998,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>M293013</t>
+          <t>M293025</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr"/>
@@ -3020,32 +3006,32 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>0815-16A</t>
+          <t>2245D-03V32</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>CONVULTED, PTFE HOSE, WITH ST/ST BRAID ANTI STATIC</t>
+          <t>MTR POLYFLEX SLANG</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>0815</t>
-        </is>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>2245D</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Dicsa</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>M293025</t>
+          <t>2245D-03V32</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -3053,17 +3039,17 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
+          <t>2248D-05V32-TC</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>MTR POLYFLEX SLANG</t>
+          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>2245D</t>
+          <t>2248D</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -3078,25 +3064,29 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>2245D-03V32</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr"/>
+          <t>2248D-05V32-TC</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>1035</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
+          <t>2380M-04V30W</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>WP. 1035 BAR / BP. 2588 BAR ID. 8.1 ±0.1 / OD. 13.4 ±0.1</t>
+          <t>PARKER POLYFLEX SLANG BLACK</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>2248D</t>
+          <t>2380M</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -3111,29 +3101,25 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>2248D-05V32-TC</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
-        <is>
-          <t>1035</t>
-        </is>
-      </c>
+          <t>2380M-04V30W</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
+          <t>2648N-32V80</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>PARKER POLYFLEX SLANG BLACK</t>
+          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>2380M</t>
+          <t>2648N</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -3148,25 +3134,29 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>2380M-04V30W</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr"/>
+          <t>2648N-32V80</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
+          <t>510A-4</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>BLACK EAGLE 2″ WP 15.000 PSI</t>
+          <t>PARFLEX 510A-4 DN06</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>2648N</t>
+          <t>510A</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -3181,29 +3171,25 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>2648N-32V80</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>510A-4</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 510A-4 DN06</t>
+          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>510A</t>
+          <t>5155</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -3218,7 +3204,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>510A-4</t>
+          <t>5155-3</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -3226,12 +3212,12 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>5155-5</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC FUEL HOSE SAE 30R3 4.3MM (3/16) DN05</t>
+          <t>PARFLEX 5155-5 DN08</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3251,7 +3237,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>5155-3</t>
+          <t>5155-5</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -3259,22 +3245,22 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
+          <t>518C-04</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX 5155-5 DN08</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>5155</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>518C</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -3284,20 +3270,24 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>5155-5</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr"/>
+          <t>518C-4</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>518C-04</t>
+          <t>518C-06</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 6.3MM (1/4) DN06 R7 WP. 190 BAR</t>
+          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -3317,34 +3307,34 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>518C-4</t>
+          <t>518C-6</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>155</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>518C-06</t>
+          <t>526BA-4</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>THERMOPLASTIC NON-CONDUCTIVE 9.5MM (3/8) DN10 R7 WP. 155 BAR</t>
+          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>518C</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>526BA</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -3354,29 +3344,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>518C-6</t>
+          <t>526BA-4</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>413,7</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
+          <t>540N-2</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>BREATHING AIR REFILL HOSE 6000 PSI CONSTANT PRESSURE</t>
+          <t>MTR NYLAFLOW HOSE R7</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>526BA</t>
+          <t>540N</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3391,19 +3381,15 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>526BA-4</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
-        <is>
-          <t>413,7</t>
-        </is>
-      </c>
+          <t>540N-2</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -3416,9 +3402,9 @@
           <t>540N</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -3428,7 +3414,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>540N-2</t>
+          <t>540N-3</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -3436,7 +3422,7 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -3461,7 +3447,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>540N-3</t>
+          <t>540N-6</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -3469,7 +3455,7 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
+          <t>540N-8</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
@@ -3494,7 +3480,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>540N-6</t>
+          <t>540N-8-DL</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -3502,22 +3488,22 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>540N-8</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>MTR NYLAFLOW HOSE R7</t>
+          <t>PARFLEX-SCHLAUCH DN12 H</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>540N</t>
-        </is>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>540P</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -3527,7 +3513,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>540N-8-DL</t>
+          <t>540P-8</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr"/>
@@ -3535,17 +3521,17 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
+          <t>56DH-2</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX-SCHLAUCH DN12 H</t>
+          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>540P</t>
+          <t>56DH</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -3560,7 +3546,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>540P-8</t>
+          <t>56DH-2</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -3568,17 +3554,17 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
+          <t>575XN-8</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>PARKER DIAGNOSTIC PLASTIC HOSE</t>
+          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>56DH</t>
+          <t>575XN</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3593,25 +3579,29 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>56DH-2</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr"/>
+          <t>575XN-8</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>344,7</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
+          <t>580N-04</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>LOW EXP./WP 5000 PSI PARFLEX</t>
+          <t>PARFLEX HOSE 580N-4</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>575XN</t>
+          <t>580N</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -3626,24 +3616,20 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>575XN-8</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>344,7</t>
-        </is>
-      </c>
+          <t>580N-4</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>580N-04</t>
+          <t>580N-06</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-4</t>
+          <t>PARFLEX HOSE 580N-6</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3663,7 +3649,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>580N-4</t>
+          <t>580N-6</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -3671,22 +3657,22 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>580N-06</t>
+          <t>588N-06</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>PARFLEX HOSE 580N-6</t>
+          <t>MTR PARFLEX SLANG R8 588N-6</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>580N</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+          <t>588N</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Alleen Staal</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3696,7 +3682,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>580N-6</t>
+          <t>588N-6</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr"/>
@@ -3704,12 +3690,12 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>588N-06</t>
+          <t>588N-4</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8 588N-6</t>
+          <t>MTR PARFLEX SLANG R8</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -3729,7 +3715,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>588N-6</t>
+          <t>588N-4</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -3737,40 +3723,44 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
+          <t>7200-04</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>MTR PARFLEX SLANG R8</t>
+          <t>HYDR. HOSE 700 BAR</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>588N</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Alleen Staal</t>
+          <t>7200</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Calseyde</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>588N-4</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="inlineStr"/>
+          <t>VHP-DN06-0412</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>7200-04</t>
+          <t>7200-06</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -3795,7 +3785,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0412</t>
+          <t>VHP-DN10-0414</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -3807,22 +3797,22 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>7200-06</t>
+          <t>7200N-04</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR</t>
+          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>7200</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>7200N</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3832,7 +3822,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN10-0414</t>
+          <t>VHP-DN06-0462</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -3844,17 +3834,17 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>7200N-04</t>
+          <t>811-56</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>HYDR. HOSE 700 BAR NON-CONDUCTIVE</t>
+          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>7200N</t>
+          <t>811</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3864,34 +3854,30 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Calseyde</t>
+          <t>Dietzel</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>VHP-DN06-0462</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
+          <t>14A-56</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>811-56</t>
+          <t>811S-32</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 89MM (3-1/2) DN90 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>811S</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -3901,25 +3887,29 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>Dietzel</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>14A-56</t>
-        </is>
-      </c>
-      <c r="G80" s="5" t="inlineStr"/>
+          <t>811S-32</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
+          <t>811S-40</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 50.8MM (2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -3927,9 +3917,9 @@
           <t>811S</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Alleen RVS</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3939,7 +3929,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>811S-32</t>
+          <t>811S-40</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -3951,12 +3941,12 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
+          <t>811S-48</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (2-1/2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -3976,7 +3966,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>811S-40</t>
+          <t>811S-48</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3988,12 +3978,12 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
+          <t>811S-56</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 76.2MM (3) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -4013,24 +4003,20 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>811S-48</t>
-        </is>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>811S-56</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>811S-64</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 88.9MM (31/2) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -4050,7 +4036,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>811S-56</t>
+          <t>811S-64</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr"/>
@@ -4058,12 +4044,12 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>811S-80</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 101.6MM (4) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -4083,7 +4069,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>811S-64</t>
+          <t>811S-80</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr"/>
@@ -4091,12 +4077,12 @@
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
+          <t>811S-96</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 127.0MM (5) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -4116,7 +4102,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>811S-80</t>
+          <t>811S-96</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr"/>
@@ -4124,22 +4110,22 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
+          <t>881-40</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 152.4MM (6) 100R4 SUCTION AND RETURN</t>
+          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>811S</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>Alleen RVS</t>
+          <t>881</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Staal + RVS</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -4149,25 +4135,29 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>811S-96</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="inlineStr"/>
+          <t>881-40</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>NO-SKIVE 63.5MM (21/2) DN63 100R4 SUCTION AND RETURN</t>
+          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>AIR06MM</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -4177,34 +4167,30 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Parker</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>881-40</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>P002228</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 ø 6x12 mm</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>AIR06MM</t>
+          <t>AIR08MM</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -4219,7 +4205,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>P002228</t>
+          <t>P002231</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr"/>
@@ -4227,17 +4213,17 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>AIR08MM</t>
+          <t>AIR10MM</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -4252,7 +4238,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>P002231</t>
+          <t>P002208</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr"/>
@@ -4260,17 +4246,17 @@
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2-ø10X17MM</t>
+          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>AIR10MM</t>
+          <t>AIR13MM</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -4285,7 +4271,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>P002208</t>
+          <t>P002211</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr"/>
@@ -4293,17 +4279,17 @@
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE AIRFORM PLW 20 Ø 13 x 21 mm</t>
+          <t>LUCHTSLANG AIRFORM BS5118/2</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>AIR13MM</t>
+          <t>AIR16MM</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -4313,12 +4299,12 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Arbon</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>P002211</t>
+          <t>5941625 L=50 mtr.</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr"/>
@@ -4326,7 +4312,7 @@
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -4336,7 +4322,7 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>AIR16MM</t>
+          <t>AIR19MM</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -4351,7 +4337,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>5941625 L=50 mtr.</t>
+          <t>5941929-NOBRA AIR L=20 mtr</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr"/>
@@ -4359,7 +4345,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -4369,7 +4355,7 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>AIR19MM</t>
+          <t>AIR25MM</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -4379,12 +4365,12 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>Arbon</t>
+          <t>Peters</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>5941929-NOBRA AIR L=20 mtr</t>
+          <t>P002223</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr"/>
@@ -4392,7 +4378,7 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -4402,7 +4388,7 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>AIR25MM</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -4417,7 +4403,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>P002223</t>
+          <t>AIR38MM</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr"/>
@@ -4425,17 +4411,17 @@
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>LUCHTSLANG AIRFORM BS5118/2</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>NOBELAIR 06X12MM</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -4450,7 +4436,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>AIR38MM</t>
+          <t>P000199</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr"/>
@@ -4458,17 +4444,17 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 06X12MM</t>
+          <t>NOBELAIR 08X13MM</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -4483,7 +4469,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>P000199</t>
+          <t>20LNBL008000079</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr"/>
@@ -4491,17 +4477,17 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>AIRHOSE NOBEL AIR BLUE SOFT</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X13MM</t>
+          <t>NOBELAIR 08X14MM</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -4516,7 +4502,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>20LNBL008000079</t>
+          <t>P000201</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr"/>
@@ -4524,7 +4510,7 @@
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -4534,7 +4520,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 08X14MM</t>
+          <t>NOBELAIR 10X16MM</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -4549,7 +4535,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>P000201</t>
+          <t>P000196</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr"/>
@@ -4557,7 +4543,7 @@
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -4567,7 +4553,7 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MM</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -4582,7 +4568,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>P000196</t>
+          <t>NOBELAIR 10X16MMRED</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr"/>
@@ -4590,7 +4576,7 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -4600,7 +4586,7 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>NOBELAIR 12X19MM</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -4615,7 +4601,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 10X16MMRED</t>
+          <t>P000197</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr"/>
@@ -4623,17 +4609,17 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 12X19MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 12X19MM</t>
+          <t>NOBELAIR 13X19MM</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -4648,7 +4634,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>P000197</t>
+          <t>20LNBL013000079</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr"/>
@@ -4656,17 +4642,17 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 13X19MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>AIR HOSE NOBEL AIR BLUE SOFT</t>
+          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 13X19MM</t>
+          <t>NOBELAIR 19X28MM</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -4681,7 +4667,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>20LNBL013000079</t>
+          <t>P000198</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr"/>
@@ -4689,17 +4675,17 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 19X28MM</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>ADEMLUCHTSLANG NOBEL AIR AS/R BREATH</t>
+          <t>PARKER HOSE 1/8″</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>NOBELAIR 19X28MM</t>
+          <t>PDH</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -4709,51 +4695,18 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>Peters</t>
+          <t>Parker</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>P000198</t>
+          <t>PDH-2</t>
         </is>
       </c>
       <c r="G104" s="5" t="inlineStr"/>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>PARKER HOSE 1/8″</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>PDH</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>Staal + RVS</t>
-        </is>
-      </c>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>Parker</t>
-        </is>
-      </c>
-      <c r="F105" s="5" t="inlineStr">
-        <is>
-          <t>PDH-2</t>
-        </is>
-      </c>
-      <c r="G105" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G105"/>
+  <autoFilter ref="A1:G104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>